<commit_message>
Auto-save: 2 file(s) — 2026-10-21 12:32
</commit_message>
<xml_diff>
--- a/Notes/2026-09-29-xloop-linkedin-blog-content-calendar-q2-v4.xlsx
+++ b/Notes/2026-09-29-xloop-linkedin-blog-content-calendar-q2-v4.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13CEF287-B6A0-4240-B08D-F9F9434C5E85}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18AE1C92-35EE-4B94-A5CD-34454F22DCCC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="24720" windowHeight="12105" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="1" r:id="rId1"/>
@@ -6670,7 +6670,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="ddd\ dd\ mmm\ yyyy"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6733,6 +6733,11 @@
       <sz val="10"/>
       <color rgb="FFB45309"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="14">
@@ -6830,7 +6835,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -6889,16 +6894,6 @@
     <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -6906,12 +6901,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7276,141 +7284,141 @@
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
     </row>
     <row r="5" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="30"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
     </row>
     <row r="7" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="22"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
     </row>
     <row r="8" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="30"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="30"/>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="22"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="30"/>
+      <c r="H12" s="30"/>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="22"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="30"/>
     </row>
     <row r="16" spans="1:8" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
@@ -7424,14 +7432,14 @@
       <c r="B17" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="23"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="29"/>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
@@ -7440,14 +7448,14 @@
       <c r="B18" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="24" t="s">
+      <c r="C18" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="24"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
@@ -7456,14 +7464,14 @@
       <c r="B19" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="24" t="s">
+      <c r="C19" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
@@ -7472,14 +7480,14 @@
       <c r="B20" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="24" t="s">
+      <c r="C20" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
@@ -7488,14 +7496,14 @@
       <c r="B21" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="24" t="s">
+      <c r="C21" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="24"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
@@ -7504,14 +7512,14 @@
       <c r="B22" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C22" s="24" t="s">
+      <c r="C22" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="24"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="27"/>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
@@ -7520,14 +7528,14 @@
       <c r="B23" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="C23" s="24" t="s">
+      <c r="C23" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="24"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
@@ -7536,14 +7544,14 @@
       <c r="B24" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C24" s="24" t="s">
+      <c r="C24" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="24"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
     </row>
     <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
@@ -7552,14 +7560,14 @@
       <c r="B25" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="24" t="s">
+      <c r="C25" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="24"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="27"/>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
@@ -7568,14 +7576,14 @@
       <c r="B26" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C26" s="24" t="s">
+      <c r="C26" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="24"/>
-      <c r="H26" s="24"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="27"/>
+      <c r="H26" s="27"/>
     </row>
     <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
@@ -7584,14 +7592,14 @@
       <c r="B27" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C27" s="24" t="s">
+      <c r="C27" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="24"/>
-      <c r="H27" s="24"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="27"/>
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
@@ -7600,14 +7608,14 @@
       <c r="B28" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C28" s="24" t="s">
+      <c r="C28" s="27" t="s">
         <v>57</v>
       </c>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="24"/>
-      <c r="H28" s="24"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="27"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="27"/>
     </row>
     <row r="30" spans="1:8" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
@@ -7618,99 +7626,99 @@
       <c r="A31" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B31" s="24" t="s">
+      <c r="B31" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="24"/>
-      <c r="F31" s="24"/>
-      <c r="G31" s="24"/>
-      <c r="H31" s="24"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="27"/>
+      <c r="E31" s="27"/>
+      <c r="F31" s="27"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="27"/>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B32" s="24" t="s">
+      <c r="B32" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="C32" s="24"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="24"/>
-      <c r="H32" s="24"/>
+      <c r="C32" s="27"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
+      <c r="F32" s="27"/>
+      <c r="G32" s="27"/>
+      <c r="H32" s="27"/>
     </row>
     <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B33" s="24" t="s">
+      <c r="B33" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
-      <c r="G33" s="24"/>
-      <c r="H33" s="24"/>
+      <c r="C33" s="27"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="27"/>
+      <c r="G33" s="27"/>
+      <c r="H33" s="27"/>
     </row>
     <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B34" s="24" t="s">
+      <c r="B34" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="C34" s="24"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="24"/>
-      <c r="H34" s="24"/>
+      <c r="C34" s="27"/>
+      <c r="D34" s="27"/>
+      <c r="E34" s="27"/>
+      <c r="F34" s="27"/>
+      <c r="G34" s="27"/>
+      <c r="H34" s="27"/>
     </row>
     <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B35" s="24" t="s">
+      <c r="B35" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="C35" s="24"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="24"/>
-      <c r="F35" s="24"/>
-      <c r="G35" s="24"/>
-      <c r="H35" s="24"/>
+      <c r="C35" s="27"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="27"/>
+      <c r="G35" s="27"/>
+      <c r="H35" s="27"/>
     </row>
     <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B36" s="24" t="s">
+      <c r="B36" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="C36" s="24"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="24"/>
-      <c r="F36" s="24"/>
-      <c r="G36" s="24"/>
-      <c r="H36" s="24"/>
+      <c r="C36" s="27"/>
+      <c r="D36" s="27"/>
+      <c r="E36" s="27"/>
+      <c r="F36" s="27"/>
+      <c r="G36" s="27"/>
+      <c r="H36" s="27"/>
     </row>
     <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B37" s="24" t="s">
+      <c r="B37" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="C37" s="24"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="24"/>
-      <c r="F37" s="24"/>
-      <c r="G37" s="24"/>
-      <c r="H37" s="24"/>
+      <c r="C37" s="27"/>
+      <c r="D37" s="27"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="27"/>
+      <c r="G37" s="27"/>
+      <c r="H37" s="27"/>
     </row>
     <row r="39" spans="1:8" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
@@ -7718,16 +7726,16 @@
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="25" t="s">
+      <c r="A40" s="28" t="s">
         <v>74</v>
       </c>
-      <c r="B40" s="25"/>
-      <c r="C40" s="25"/>
-      <c r="D40" s="25"/>
-      <c r="E40" s="25"/>
-      <c r="F40" s="25"/>
-      <c r="G40" s="25"/>
-      <c r="H40" s="25"/>
+      <c r="B40" s="28"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="28"/>
+      <c r="E40" s="28"/>
+      <c r="F40" s="28"/>
+      <c r="G40" s="28"/>
+      <c r="H40" s="28"/>
     </row>
     <row r="42" spans="1:8" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
@@ -7735,28 +7743,28 @@
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="26" t="s">
+      <c r="A43" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="B43" s="26"/>
+      <c r="B43" s="22"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="27" t="s">
+      <c r="A44" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="B44" s="27"/>
+      <c r="B44" s="23"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="28" t="s">
+      <c r="A45" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="B45" s="28"/>
+      <c r="B45" s="24"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="29" t="s">
+      <c r="A46" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="B46" s="29"/>
+      <c r="B46" s="25"/>
     </row>
     <row r="48" spans="1:8" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
@@ -7764,54 +7772,54 @@
       </c>
     </row>
     <row r="49" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="30" t="s">
+      <c r="A49" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="B49" s="30"/>
-      <c r="C49" s="30"/>
-      <c r="D49" s="30"/>
-      <c r="E49" s="30"/>
-      <c r="F49" s="30"/>
-      <c r="G49" s="30"/>
-      <c r="H49" s="30"/>
+      <c r="B49" s="26"/>
+      <c r="C49" s="26"/>
+      <c r="D49" s="26"/>
+      <c r="E49" s="26"/>
+      <c r="F49" s="26"/>
+      <c r="G49" s="26"/>
+      <c r="H49" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="35">
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="B8:H8"/>
+    <mergeCell ref="B9:H9"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="C17:H17"/>
+    <mergeCell ref="C18:H18"/>
+    <mergeCell ref="C19:H19"/>
+    <mergeCell ref="C20:H20"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
+    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C26:H26"/>
+    <mergeCell ref="C27:H27"/>
+    <mergeCell ref="C28:H28"/>
+    <mergeCell ref="B31:H31"/>
+    <mergeCell ref="B32:H32"/>
+    <mergeCell ref="B33:H33"/>
+    <mergeCell ref="B34:H34"/>
+    <mergeCell ref="B35:H35"/>
+    <mergeCell ref="B36:H36"/>
+    <mergeCell ref="B37:H37"/>
+    <mergeCell ref="A40:H40"/>
     <mergeCell ref="A43:B43"/>
     <mergeCell ref="A44:B44"/>
     <mergeCell ref="A45:B45"/>
     <mergeCell ref="A46:B46"/>
     <mergeCell ref="A49:H49"/>
-    <mergeCell ref="B34:H34"/>
-    <mergeCell ref="B35:H35"/>
-    <mergeCell ref="B36:H36"/>
-    <mergeCell ref="B37:H37"/>
-    <mergeCell ref="A40:H40"/>
-    <mergeCell ref="C27:H27"/>
-    <mergeCell ref="C28:H28"/>
-    <mergeCell ref="B31:H31"/>
-    <mergeCell ref="B32:H32"/>
-    <mergeCell ref="B33:H33"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C23:H23"/>
-    <mergeCell ref="C24:H24"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C26:H26"/>
-    <mergeCell ref="C17:H17"/>
-    <mergeCell ref="C18:H18"/>
-    <mergeCell ref="C19:H19"/>
-    <mergeCell ref="C20:H20"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="B9:H9"/>
-    <mergeCell ref="B10:H10"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="B7:H7"/>
-    <mergeCell ref="B8:H8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
@@ -7861,16 +7869,16 @@
       <c r="B4" s="33"/>
       <c r="C4" s="33"/>
       <c r="D4" s="33"/>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="30" t="s">
         <v>1538</v>
       </c>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
     </row>
     <row r="5" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
@@ -7879,16 +7887,16 @@
       <c r="B5" s="33"/>
       <c r="C5" s="33"/>
       <c r="D5" s="33"/>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="30" t="s">
         <v>1539</v>
       </c>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="30"/>
+      <c r="L5" s="30"/>
     </row>
     <row r="6" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
@@ -7897,16 +7905,16 @@
       <c r="B6" s="33"/>
       <c r="C6" s="33"/>
       <c r="D6" s="33"/>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="30" t="s">
         <v>1540</v>
       </c>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="30"/>
+      <c r="K6" s="30"/>
+      <c r="L6" s="30"/>
     </row>
     <row r="7" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
@@ -7915,16 +7923,16 @@
       <c r="B7" s="33"/>
       <c r="C7" s="33"/>
       <c r="D7" s="33"/>
-      <c r="E7" s="22" t="s">
+      <c r="E7" s="30" t="s">
         <v>1541</v>
       </c>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+      <c r="J7" s="30"/>
+      <c r="K7" s="30"/>
+      <c r="L7" s="30"/>
     </row>
     <row r="8" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
@@ -7933,16 +7941,16 @@
       <c r="B8" s="33"/>
       <c r="C8" s="33"/>
       <c r="D8" s="33"/>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="30" t="s">
         <v>1542</v>
       </c>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="22"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="30"/>
     </row>
     <row r="9" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
@@ -7951,16 +7959,16 @@
       <c r="B9" s="33"/>
       <c r="C9" s="33"/>
       <c r="D9" s="33"/>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="30" t="s">
         <v>1543</v>
       </c>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="22"/>
-      <c r="L9" s="22"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30"/>
+      <c r="K9" s="30"/>
+      <c r="L9" s="30"/>
     </row>
     <row r="10" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
@@ -7969,16 +7977,16 @@
       <c r="B10" s="33"/>
       <c r="C10" s="33"/>
       <c r="D10" s="33"/>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="30" t="s">
         <v>1254</v>
       </c>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="22"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="12" spans="1:22" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
@@ -8867,6 +8875,12 @@
   </sheetData>
   <autoFilter ref="A12:V24" xr:uid="{00000000-0009-0000-0000-000009000000}"/>
   <mergeCells count="14">
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:L4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E5:L5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:L6"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="E10:L10"/>
     <mergeCell ref="A7:D7"/>
@@ -8875,12 +8889,6 @@
     <mergeCell ref="E8:L8"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="E9:L9"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:L4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:L5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="E6:L6"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="U13:U24" xr:uid="{00000000-0002-0000-0900-000000000000}">
@@ -8935,16 +8943,16 @@
       <c r="B4" s="33"/>
       <c r="C4" s="33"/>
       <c r="D4" s="33"/>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="30" t="s">
         <v>1601</v>
       </c>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
     </row>
     <row r="5" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
@@ -8953,16 +8961,16 @@
       <c r="B5" s="33"/>
       <c r="C5" s="33"/>
       <c r="D5" s="33"/>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="30" t="s">
         <v>1602</v>
       </c>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="30"/>
+      <c r="L5" s="30"/>
     </row>
     <row r="6" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
@@ -8971,16 +8979,16 @@
       <c r="B6" s="33"/>
       <c r="C6" s="33"/>
       <c r="D6" s="33"/>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="30" t="s">
         <v>1603</v>
       </c>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="30"/>
+      <c r="K6" s="30"/>
+      <c r="L6" s="30"/>
     </row>
     <row r="7" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
@@ -8989,16 +8997,16 @@
       <c r="B7" s="33"/>
       <c r="C7" s="33"/>
       <c r="D7" s="33"/>
-      <c r="E7" s="22" t="s">
+      <c r="E7" s="30" t="s">
         <v>1604</v>
       </c>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+      <c r="J7" s="30"/>
+      <c r="K7" s="30"/>
+      <c r="L7" s="30"/>
     </row>
     <row r="8" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
@@ -9007,16 +9015,16 @@
       <c r="B8" s="33"/>
       <c r="C8" s="33"/>
       <c r="D8" s="33"/>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="30" t="s">
         <v>1605</v>
       </c>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="22"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="30"/>
     </row>
     <row r="9" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
@@ -9025,16 +9033,16 @@
       <c r="B9" s="33"/>
       <c r="C9" s="33"/>
       <c r="D9" s="33"/>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="30" t="s">
         <v>1606</v>
       </c>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="22"/>
-      <c r="L9" s="22"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30"/>
+      <c r="K9" s="30"/>
+      <c r="L9" s="30"/>
     </row>
     <row r="10" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
@@ -9043,16 +9051,16 @@
       <c r="B10" s="33"/>
       <c r="C10" s="33"/>
       <c r="D10" s="33"/>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="30" t="s">
         <v>1254</v>
       </c>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="22"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="12" spans="1:22" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
@@ -10213,6 +10221,12 @@
   </sheetData>
   <autoFilter ref="A12:V28" xr:uid="{00000000-0009-0000-0000-00000A000000}"/>
   <mergeCells count="14">
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:L4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E5:L5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:L6"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="E10:L10"/>
     <mergeCell ref="A7:D7"/>
@@ -10221,12 +10235,6 @@
     <mergeCell ref="E8:L8"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="E9:L9"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:L4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:L5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="E6:L6"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="U13:U28" xr:uid="{00000000-0002-0000-0A00-000000000000}">
@@ -10624,12 +10632,12 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="32" t="s">
         <v>1732</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
     </row>
     <row r="6" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
@@ -10836,61 +10844,61 @@
       <c r="A22" s="6" t="s">
         <v>323</v>
       </c>
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="27" t="s">
         <v>1754</v>
       </c>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
     </row>
     <row r="23" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>1755</v>
       </c>
-      <c r="B23" s="24" t="s">
+      <c r="B23" s="27" t="s">
         <v>1756</v>
       </c>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
     </row>
     <row r="24" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>1757</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="27" t="s">
         <v>1758</v>
       </c>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
     </row>
     <row r="25" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>1759</v>
       </c>
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="27" t="s">
         <v>1760</v>
       </c>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
     </row>
     <row r="26" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>366</v>
       </c>
-      <c r="B26" s="24" t="s">
+      <c r="B26" s="27" t="s">
         <v>1761</v>
       </c>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="27"/>
     </row>
     <row r="27" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>1762</v>
       </c>
-      <c r="B27" s="24" t="s">
+      <c r="B27" s="27" t="s">
         <v>1763</v>
       </c>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
     </row>
     <row r="29" spans="1:4" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
@@ -10901,61 +10909,61 @@
       <c r="A30" t="s">
         <v>308</v>
       </c>
-      <c r="B30" s="31" t="s">
+      <c r="B30" s="32" t="s">
         <v>1765</v>
       </c>
-      <c r="C30" s="31"/>
-      <c r="D30" s="31"/>
+      <c r="C30" s="32"/>
+      <c r="D30" s="32"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>308</v>
       </c>
-      <c r="B31" s="31" t="s">
+      <c r="B31" s="32" t="s">
         <v>1766</v>
       </c>
-      <c r="C31" s="31"/>
-      <c r="D31" s="31"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="32"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>308</v>
       </c>
-      <c r="B32" s="31" t="s">
+      <c r="B32" s="32" t="s">
         <v>1767</v>
       </c>
-      <c r="C32" s="31"/>
-      <c r="D32" s="31"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>308</v>
       </c>
-      <c r="B33" s="31" t="s">
+      <c r="B33" s="32" t="s">
         <v>1768</v>
       </c>
-      <c r="C33" s="31"/>
-      <c r="D33" s="31"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>308</v>
       </c>
-      <c r="B34" s="31" t="s">
+      <c r="B34" s="32" t="s">
         <v>1769</v>
       </c>
-      <c r="C34" s="31"/>
-      <c r="D34" s="31"/>
+      <c r="C34" s="32"/>
+      <c r="D34" s="32"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>308</v>
       </c>
-      <c r="B35" s="31" t="s">
+      <c r="B35" s="32" t="s">
         <v>1770</v>
       </c>
-      <c r="C35" s="31"/>
-      <c r="D35" s="31"/>
+      <c r="C35" s="32"/>
+      <c r="D35" s="32"/>
     </row>
     <row r="37" spans="1:4" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
@@ -10963,15 +10971,20 @@
       </c>
     </row>
     <row r="38" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="31" t="s">
+      <c r="A38" s="32" t="s">
         <v>1772</v>
       </c>
-      <c r="B38" s="31"/>
-      <c r="C38" s="31"/>
-      <c r="D38" s="31"/>
+      <c r="B38" s="32"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B25:D25"/>
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="B34:D34"/>
     <mergeCell ref="B35:D35"/>
@@ -10981,11 +10994,6 @@
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B31:D31"/>
     <mergeCell ref="B32:D32"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="B25:D25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
@@ -11327,132 +11335,138 @@
       <c r="A21" s="6" t="s">
         <v>1849</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="27" t="s">
         <v>1850</v>
       </c>
-      <c r="C21" s="24"/>
+      <c r="C21" s="27"/>
       <c r="D21" s="6" t="s">
         <v>1851</v>
       </c>
-      <c r="E21" s="24" t="s">
+      <c r="E21" s="27" t="s">
         <v>1852</v>
       </c>
-      <c r="F21" s="24"/>
+      <c r="F21" s="27"/>
     </row>
     <row r="22" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>1853</v>
       </c>
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="27" t="s">
         <v>1854</v>
       </c>
-      <c r="C22" s="24"/>
+      <c r="C22" s="27"/>
       <c r="D22" s="6" t="s">
         <v>1855</v>
       </c>
-      <c r="E22" s="24" t="s">
+      <c r="E22" s="27" t="s">
         <v>1856</v>
       </c>
-      <c r="F22" s="24"/>
+      <c r="F22" s="27"/>
     </row>
     <row r="23" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>1857</v>
       </c>
-      <c r="B23" s="24" t="s">
+      <c r="B23" s="27" t="s">
         <v>1283</v>
       </c>
-      <c r="C23" s="24"/>
+      <c r="C23" s="27"/>
       <c r="D23" s="6" t="s">
         <v>1858</v>
       </c>
-      <c r="E23" s="24" t="s">
+      <c r="E23" s="27" t="s">
         <v>1859</v>
       </c>
-      <c r="F23" s="24"/>
+      <c r="F23" s="27"/>
     </row>
     <row r="24" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>1860</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="27" t="s">
         <v>1861</v>
       </c>
-      <c r="C24" s="24"/>
+      <c r="C24" s="27"/>
       <c r="D24" s="6" t="s">
         <v>1862</v>
       </c>
-      <c r="E24" s="24" t="s">
+      <c r="E24" s="27" t="s">
         <v>1863</v>
       </c>
-      <c r="F24" s="24"/>
+      <c r="F24" s="27"/>
     </row>
     <row r="25" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>1864</v>
       </c>
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="27" t="s">
         <v>1865</v>
       </c>
-      <c r="C25" s="24"/>
+      <c r="C25" s="27"/>
       <c r="D25" s="6" t="s">
         <v>1866</v>
       </c>
-      <c r="E25" s="24" t="s">
+      <c r="E25" s="27" t="s">
         <v>1867</v>
       </c>
-      <c r="F25" s="24"/>
+      <c r="F25" s="27"/>
     </row>
     <row r="26" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>1868</v>
       </c>
-      <c r="B26" s="24" t="s">
+      <c r="B26" s="27" t="s">
         <v>1869</v>
       </c>
-      <c r="C26" s="24"/>
+      <c r="C26" s="27"/>
       <c r="D26" s="6" t="s">
         <v>1870</v>
       </c>
-      <c r="E26" s="24" t="s">
+      <c r="E26" s="27" t="s">
         <v>1871</v>
       </c>
-      <c r="F26" s="24"/>
+      <c r="F26" s="27"/>
     </row>
     <row r="27" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>1872</v>
       </c>
-      <c r="B27" s="24" t="s">
+      <c r="B27" s="27" t="s">
         <v>1873</v>
       </c>
-      <c r="C27" s="24"/>
+      <c r="C27" s="27"/>
       <c r="D27" s="6" t="s">
         <v>1874</v>
       </c>
-      <c r="E27" s="24" t="s">
+      <c r="E27" s="27" t="s">
         <v>1875</v>
       </c>
-      <c r="F27" s="24"/>
+      <c r="F27" s="27"/>
     </row>
     <row r="28" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>1876</v>
       </c>
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="27" t="s">
         <v>1877</v>
       </c>
-      <c r="C28" s="24"/>
+      <c r="C28" s="27"/>
       <c r="D28" s="6" t="s">
         <v>1878</v>
       </c>
-      <c r="E28" s="24" t="s">
+      <c r="E28" s="27" t="s">
         <v>1879</v>
       </c>
-      <c r="F28" s="24"/>
+      <c r="F28" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="E23:F23"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="E27:F27"/>
     <mergeCell ref="B28:C28"/>
@@ -11463,12 +11477,6 @@
     <mergeCell ref="E25:F25"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="E26:F26"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="E23:F23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
@@ -13632,79 +13640,79 @@
       <c r="A18" t="s">
         <v>308</v>
       </c>
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="32" t="s">
         <v>309</v>
       </c>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="31"/>
-      <c r="G18" s="31"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="32"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>308</v>
       </c>
-      <c r="B19" s="31" t="s">
+      <c r="B19" s="32" t="s">
         <v>310</v>
       </c>
-      <c r="C19" s="31"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="31"/>
-      <c r="G19" s="31"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>308</v>
       </c>
-      <c r="B20" s="31" t="s">
+      <c r="B20" s="32" t="s">
         <v>311</v>
       </c>
-      <c r="C20" s="31"/>
-      <c r="D20" s="31"/>
-      <c r="E20" s="31"/>
-      <c r="F20" s="31"/>
-      <c r="G20" s="31"/>
+      <c r="C20" s="32"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>308</v>
       </c>
-      <c r="B21" s="31" t="s">
+      <c r="B21" s="32" t="s">
         <v>312</v>
       </c>
-      <c r="C21" s="31"/>
-      <c r="D21" s="31"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="31"/>
-      <c r="G21" s="31"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>308</v>
       </c>
-      <c r="B22" s="31" t="s">
+      <c r="B22" s="32" t="s">
         <v>313</v>
       </c>
-      <c r="C22" s="31"/>
-      <c r="D22" s="31"/>
-      <c r="E22" s="31"/>
-      <c r="F22" s="31"/>
-      <c r="G22" s="31"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>308</v>
       </c>
-      <c r="B23" s="31" t="s">
+      <c r="B23" s="32" t="s">
         <v>314</v>
       </c>
-      <c r="C23" s="31"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="31"/>
-      <c r="F23" s="31"/>
-      <c r="G23" s="31"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="32"/>
+      <c r="G23" s="32"/>
     </row>
     <row r="25" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
@@ -13712,68 +13720,68 @@
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B26" s="32" t="s">
+      <c r="B26" s="31" t="s">
         <v>316</v>
       </c>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B27" s="32" t="s">
+      <c r="B27" s="31" t="s">
         <v>317</v>
       </c>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="32"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31"/>
+      <c r="G27" s="31"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B28" s="32" t="s">
+      <c r="B28" s="31" t="s">
         <v>318</v>
       </c>
-      <c r="C28" s="32"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="31"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B29" s="32" t="s">
+      <c r="B29" s="31" t="s">
         <v>319</v>
       </c>
-      <c r="C29" s="32"/>
-      <c r="D29" s="32"/>
-      <c r="E29" s="32"/>
-      <c r="F29" s="32"/>
-      <c r="G29" s="32"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="31"/>
+      <c r="G29" s="31"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B30" s="32" t="s">
+      <c r="B30" s="31" t="s">
         <v>320</v>
       </c>
-      <c r="C30" s="32"/>
-      <c r="D30" s="32"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="31"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="31"/>
+      <c r="G30" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="B22:G22"/>
     <mergeCell ref="B30:G30"/>
     <mergeCell ref="B23:G23"/>
     <mergeCell ref="B26:G26"/>
     <mergeCell ref="B27:G27"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:G29"/>
-    <mergeCell ref="B18:G18"/>
-    <mergeCell ref="B19:G19"/>
-    <mergeCell ref="B20:G20"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="B22:G22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
@@ -14071,7 +14079,7 @@
       <c r="F12" s="15" t="s">
         <v>396</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="G12" s="34" t="s">
         <v>397</v>
       </c>
       <c r="H12" s="6" t="s">
@@ -15217,161 +15225,161 @@
       <c r="A31" t="s">
         <v>621</v>
       </c>
-      <c r="B31" s="31" t="s">
+      <c r="B31" s="32" t="s">
         <v>622</v>
       </c>
-      <c r="C31" s="31"/>
-      <c r="D31" s="31"/>
-      <c r="E31" s="31"/>
-      <c r="F31" s="31"/>
-      <c r="G31" s="31"/>
-      <c r="H31" s="31"/>
-      <c r="I31" s="31"/>
-      <c r="J31" s="31"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="32"/>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>621</v>
       </c>
-      <c r="B32" s="31" t="s">
+      <c r="B32" s="32" t="s">
         <v>623</v>
       </c>
-      <c r="C32" s="31"/>
-      <c r="D32" s="31"/>
-      <c r="E32" s="31"/>
-      <c r="F32" s="31"/>
-      <c r="G32" s="31"/>
-      <c r="H32" s="31"/>
-      <c r="I32" s="31"/>
-      <c r="J32" s="31"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="32"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>621</v>
       </c>
-      <c r="B33" s="31" t="s">
+      <c r="B33" s="32" t="s">
         <v>624</v>
       </c>
-      <c r="C33" s="31"/>
-      <c r="D33" s="31"/>
-      <c r="E33" s="31"/>
-      <c r="F33" s="31"/>
-      <c r="G33" s="31"/>
-      <c r="H33" s="31"/>
-      <c r="I33" s="31"/>
-      <c r="J33" s="31"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="32"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>621</v>
       </c>
-      <c r="B34" s="31" t="s">
+      <c r="B34" s="32" t="s">
         <v>625</v>
       </c>
-      <c r="C34" s="31"/>
-      <c r="D34" s="31"/>
-      <c r="E34" s="31"/>
-      <c r="F34" s="31"/>
-      <c r="G34" s="31"/>
-      <c r="H34" s="31"/>
-      <c r="I34" s="31"/>
-      <c r="J34" s="31"/>
+      <c r="C34" s="32"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="32"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>621</v>
       </c>
-      <c r="B35" s="31" t="s">
+      <c r="B35" s="32" t="s">
         <v>626</v>
       </c>
-      <c r="C35" s="31"/>
-      <c r="D35" s="31"/>
-      <c r="E35" s="31"/>
-      <c r="F35" s="31"/>
-      <c r="G35" s="31"/>
-      <c r="H35" s="31"/>
-      <c r="I35" s="31"/>
-      <c r="J35" s="31"/>
+      <c r="C35" s="32"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="32"/>
+      <c r="G35" s="32"/>
+      <c r="H35" s="32"/>
+      <c r="I35" s="32"/>
+      <c r="J35" s="32"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>621</v>
       </c>
-      <c r="B36" s="31" t="s">
+      <c r="B36" s="32" t="s">
         <v>627</v>
       </c>
-      <c r="C36" s="31"/>
-      <c r="D36" s="31"/>
-      <c r="E36" s="31"/>
-      <c r="F36" s="31"/>
-      <c r="G36" s="31"/>
-      <c r="H36" s="31"/>
-      <c r="I36" s="31"/>
-      <c r="J36" s="31"/>
+      <c r="C36" s="32"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="32"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>621</v>
       </c>
-      <c r="B37" s="31" t="s">
+      <c r="B37" s="32" t="s">
         <v>628</v>
       </c>
-      <c r="C37" s="31"/>
-      <c r="D37" s="31"/>
-      <c r="E37" s="31"/>
-      <c r="F37" s="31"/>
-      <c r="G37" s="31"/>
-      <c r="H37" s="31"/>
-      <c r="I37" s="31"/>
-      <c r="J37" s="31"/>
+      <c r="C37" s="32"/>
+      <c r="D37" s="32"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="32"/>
+      <c r="J37" s="32"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>621</v>
       </c>
-      <c r="B38" s="31" t="s">
+      <c r="B38" s="32" t="s">
         <v>629</v>
       </c>
-      <c r="C38" s="31"/>
-      <c r="D38" s="31"/>
-      <c r="E38" s="31"/>
-      <c r="F38" s="31"/>
-      <c r="G38" s="31"/>
-      <c r="H38" s="31"/>
-      <c r="I38" s="31"/>
-      <c r="J38" s="31"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="32"/>
+      <c r="J38" s="32"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>621</v>
       </c>
-      <c r="B39" s="31" t="s">
+      <c r="B39" s="32" t="s">
         <v>630</v>
       </c>
-      <c r="C39" s="31"/>
-      <c r="D39" s="31"/>
-      <c r="E39" s="31"/>
-      <c r="F39" s="31"/>
-      <c r="G39" s="31"/>
-      <c r="H39" s="31"/>
-      <c r="I39" s="31"/>
-      <c r="J39" s="31"/>
+      <c r="C39" s="32"/>
+      <c r="D39" s="32"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="32"/>
+      <c r="I39" s="32"/>
+      <c r="J39" s="32"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>621</v>
       </c>
-      <c r="B40" s="31" t="s">
+      <c r="B40" s="32" t="s">
         <v>631</v>
       </c>
-      <c r="C40" s="31"/>
-      <c r="D40" s="31"/>
-      <c r="E40" s="31"/>
-      <c r="F40" s="31"/>
-      <c r="G40" s="31"/>
-      <c r="H40" s="31"/>
-      <c r="I40" s="31"/>
-      <c r="J40" s="31"/>
+      <c r="C40" s="32"/>
+      <c r="D40" s="32"/>
+      <c r="E40" s="32"/>
+      <c r="F40" s="32"/>
+      <c r="G40" s="32"/>
+      <c r="H40" s="32"/>
+      <c r="I40" s="32"/>
+      <c r="J40" s="32"/>
     </row>
     <row r="42" spans="1:10" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
@@ -15379,167 +15387,183 @@
       </c>
     </row>
     <row r="43" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="23" t="s">
+      <c r="A43" s="29" t="s">
         <v>633</v>
       </c>
-      <c r="B43" s="23"/>
-      <c r="C43" s="23"/>
+      <c r="B43" s="29"/>
+      <c r="C43" s="29"/>
       <c r="D43" s="5" t="s">
         <v>375</v>
       </c>
       <c r="E43" s="5" t="s">
         <v>634</v>
       </c>
-      <c r="F43" s="23" t="s">
+      <c r="F43" s="29" t="s">
         <v>635</v>
       </c>
-      <c r="G43" s="23"/>
-      <c r="H43" s="23"/>
-      <c r="I43" s="23"/>
-      <c r="J43" s="23"/>
+      <c r="G43" s="29"/>
+      <c r="H43" s="29"/>
+      <c r="I43" s="29"/>
+      <c r="J43" s="29"/>
     </row>
     <row r="44" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="24" t="s">
+      <c r="A44" s="27" t="s">
         <v>636</v>
       </c>
-      <c r="B44" s="24"/>
-      <c r="C44" s="24"/>
+      <c r="B44" s="27"/>
+      <c r="C44" s="27"/>
       <c r="D44" s="6" t="s">
         <v>637</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>638</v>
       </c>
-      <c r="F44" s="24" t="s">
+      <c r="F44" s="27" t="s">
         <v>639</v>
       </c>
-      <c r="G44" s="24"/>
-      <c r="H44" s="24"/>
-      <c r="I44" s="24"/>
-      <c r="J44" s="24"/>
+      <c r="G44" s="27"/>
+      <c r="H44" s="27"/>
+      <c r="I44" s="27"/>
+      <c r="J44" s="27"/>
     </row>
     <row r="45" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="24" t="s">
+      <c r="A45" s="27" t="s">
         <v>640</v>
       </c>
-      <c r="B45" s="24"/>
-      <c r="C45" s="24"/>
+      <c r="B45" s="27"/>
+      <c r="C45" s="27"/>
       <c r="D45" s="6" t="s">
         <v>637</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>641</v>
       </c>
-      <c r="F45" s="24" t="s">
+      <c r="F45" s="27" t="s">
         <v>642</v>
       </c>
-      <c r="G45" s="24"/>
-      <c r="H45" s="24"/>
-      <c r="I45" s="24"/>
-      <c r="J45" s="24"/>
+      <c r="G45" s="27"/>
+      <c r="H45" s="27"/>
+      <c r="I45" s="27"/>
+      <c r="J45" s="27"/>
     </row>
     <row r="46" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="24" t="s">
+      <c r="A46" s="27" t="s">
         <v>643</v>
       </c>
-      <c r="B46" s="24"/>
-      <c r="C46" s="24"/>
+      <c r="B46" s="27"/>
+      <c r="C46" s="27"/>
       <c r="D46" s="6" t="s">
         <v>637</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="F46" s="24" t="s">
+      <c r="F46" s="27" t="s">
         <v>644</v>
       </c>
-      <c r="G46" s="24"/>
-      <c r="H46" s="24"/>
-      <c r="I46" s="24"/>
-      <c r="J46" s="24"/>
+      <c r="G46" s="27"/>
+      <c r="H46" s="27"/>
+      <c r="I46" s="27"/>
+      <c r="J46" s="27"/>
     </row>
     <row r="47" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="24" t="s">
+      <c r="A47" s="27" t="s">
         <v>645</v>
       </c>
-      <c r="B47" s="24"/>
-      <c r="C47" s="24"/>
+      <c r="B47" s="27"/>
+      <c r="C47" s="27"/>
       <c r="D47" s="6" t="s">
         <v>646</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="F47" s="24" t="s">
+      <c r="F47" s="27" t="s">
         <v>647</v>
       </c>
-      <c r="G47" s="24"/>
-      <c r="H47" s="24"/>
-      <c r="I47" s="24"/>
-      <c r="J47" s="24"/>
+      <c r="G47" s="27"/>
+      <c r="H47" s="27"/>
+      <c r="I47" s="27"/>
+      <c r="J47" s="27"/>
     </row>
     <row r="48" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="24" t="s">
+      <c r="A48" s="27" t="s">
         <v>648</v>
       </c>
-      <c r="B48" s="24"/>
-      <c r="C48" s="24"/>
+      <c r="B48" s="27"/>
+      <c r="C48" s="27"/>
       <c r="D48" s="6" t="s">
         <v>649</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="F48" s="24" t="s">
+      <c r="F48" s="27" t="s">
         <v>650</v>
       </c>
-      <c r="G48" s="24"/>
-      <c r="H48" s="24"/>
-      <c r="I48" s="24"/>
-      <c r="J48" s="24"/>
+      <c r="G48" s="27"/>
+      <c r="H48" s="27"/>
+      <c r="I48" s="27"/>
+      <c r="J48" s="27"/>
     </row>
     <row r="49" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="24" t="s">
+      <c r="A49" s="27" t="s">
         <v>651</v>
       </c>
-      <c r="B49" s="24"/>
-      <c r="C49" s="24"/>
+      <c r="B49" s="27"/>
+      <c r="C49" s="27"/>
       <c r="D49" s="6" t="s">
         <v>652</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="F49" s="24" t="s">
+      <c r="F49" s="27" t="s">
         <v>653</v>
       </c>
-      <c r="G49" s="24"/>
-      <c r="H49" s="24"/>
-      <c r="I49" s="24"/>
-      <c r="J49" s="24"/>
+      <c r="G49" s="27"/>
+      <c r="H49" s="27"/>
+      <c r="I49" s="27"/>
+      <c r="J49" s="27"/>
     </row>
     <row r="50" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="24" t="s">
+      <c r="A50" s="27" t="s">
         <v>654</v>
       </c>
-      <c r="B50" s="24"/>
-      <c r="C50" s="24"/>
+      <c r="B50" s="27"/>
+      <c r="C50" s="27"/>
       <c r="D50" s="6" t="s">
         <v>655</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="F50" s="24" t="s">
+      <c r="F50" s="27" t="s">
         <v>656</v>
       </c>
-      <c r="G50" s="24"/>
-      <c r="H50" s="24"/>
-      <c r="I50" s="24"/>
-      <c r="J50" s="24"/>
+      <c r="G50" s="27"/>
+      <c r="H50" s="27"/>
+      <c r="I50" s="27"/>
+      <c r="J50" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="B31:J31"/>
+    <mergeCell ref="B32:J32"/>
+    <mergeCell ref="B33:J33"/>
+    <mergeCell ref="B34:J34"/>
+    <mergeCell ref="B35:J35"/>
+    <mergeCell ref="B36:J36"/>
+    <mergeCell ref="B37:J37"/>
+    <mergeCell ref="B38:J38"/>
+    <mergeCell ref="B39:J39"/>
+    <mergeCell ref="B40:J40"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="F43:J43"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="F44:J44"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="F45:J45"/>
     <mergeCell ref="A49:C49"/>
     <mergeCell ref="F49:J49"/>
     <mergeCell ref="A50:C50"/>
@@ -15550,22 +15574,6 @@
     <mergeCell ref="F47:J47"/>
     <mergeCell ref="A48:C48"/>
     <mergeCell ref="F48:J48"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="F43:J43"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="F44:J44"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="F45:J45"/>
-    <mergeCell ref="B36:J36"/>
-    <mergeCell ref="B37:J37"/>
-    <mergeCell ref="B38:J38"/>
-    <mergeCell ref="B39:J39"/>
-    <mergeCell ref="B40:J40"/>
-    <mergeCell ref="B31:J31"/>
-    <mergeCell ref="B32:J32"/>
-    <mergeCell ref="B33:J33"/>
-    <mergeCell ref="B34:J34"/>
-    <mergeCell ref="B35:J35"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="V12:V28" xr:uid="{00000000-0002-0000-0300-000000000000}">
@@ -15573,7 +15581,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup fitToHeight="0" orientation="landscape"/>
+  <pageSetup fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -15723,7 +15731,7 @@
       <c r="F6" s="6" t="s">
         <v>682</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="34" t="s">
         <v>683</v>
       </c>
       <c r="H6" s="6" t="s">
@@ -19790,16 +19798,16 @@
       <c r="B4" s="33"/>
       <c r="C4" s="33"/>
       <c r="D4" s="33"/>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="30" t="s">
         <v>1242</v>
       </c>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
     </row>
     <row r="5" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
@@ -19808,16 +19816,16 @@
       <c r="B5" s="33"/>
       <c r="C5" s="33"/>
       <c r="D5" s="33"/>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="30" t="s">
         <v>1244</v>
       </c>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="30"/>
+      <c r="L5" s="30"/>
     </row>
     <row r="6" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
@@ -19826,16 +19834,16 @@
       <c r="B6" s="33"/>
       <c r="C6" s="33"/>
       <c r="D6" s="33"/>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="30" t="s">
         <v>1246</v>
       </c>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="30"/>
+      <c r="K6" s="30"/>
+      <c r="L6" s="30"/>
     </row>
     <row r="7" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
@@ -19844,16 +19852,16 @@
       <c r="B7" s="33"/>
       <c r="C7" s="33"/>
       <c r="D7" s="33"/>
-      <c r="E7" s="22" t="s">
+      <c r="E7" s="30" t="s">
         <v>1248</v>
       </c>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+      <c r="J7" s="30"/>
+      <c r="K7" s="30"/>
+      <c r="L7" s="30"/>
     </row>
     <row r="8" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
@@ -19862,16 +19870,16 @@
       <c r="B8" s="33"/>
       <c r="C8" s="33"/>
       <c r="D8" s="33"/>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="30" t="s">
         <v>1250</v>
       </c>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="22"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="30"/>
     </row>
     <row r="9" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
@@ -19880,16 +19888,16 @@
       <c r="B9" s="33"/>
       <c r="C9" s="33"/>
       <c r="D9" s="33"/>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="30" t="s">
         <v>1252</v>
       </c>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="22"/>
-      <c r="L9" s="22"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30"/>
+      <c r="K9" s="30"/>
+      <c r="L9" s="30"/>
     </row>
     <row r="10" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
@@ -19898,16 +19906,16 @@
       <c r="B10" s="33"/>
       <c r="C10" s="33"/>
       <c r="D10" s="33"/>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="30" t="s">
         <v>1254</v>
       </c>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="22"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="12" spans="1:22" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
@@ -20864,6 +20872,12 @@
   </sheetData>
   <autoFilter ref="A12:V25" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <mergeCells count="14">
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:L4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E5:L5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:L6"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="E10:L10"/>
     <mergeCell ref="A7:D7"/>
@@ -20872,12 +20886,6 @@
     <mergeCell ref="E8:L8"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="E9:L9"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:L4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:L5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="E6:L6"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="U13:U25" xr:uid="{00000000-0002-0000-0600-000000000000}">
@@ -20932,16 +20940,16 @@
       <c r="B4" s="33"/>
       <c r="C4" s="33"/>
       <c r="D4" s="33"/>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="30" t="s">
         <v>1352</v>
       </c>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
     </row>
     <row r="5" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
@@ -20950,16 +20958,16 @@
       <c r="B5" s="33"/>
       <c r="C5" s="33"/>
       <c r="D5" s="33"/>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="30" t="s">
         <v>1353</v>
       </c>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="30"/>
+      <c r="L5" s="30"/>
     </row>
     <row r="6" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
@@ -20968,16 +20976,16 @@
       <c r="B6" s="33"/>
       <c r="C6" s="33"/>
       <c r="D6" s="33"/>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="30" t="s">
         <v>1354</v>
       </c>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="30"/>
+      <c r="K6" s="30"/>
+      <c r="L6" s="30"/>
     </row>
     <row r="7" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
@@ -20986,16 +20994,16 @@
       <c r="B7" s="33"/>
       <c r="C7" s="33"/>
       <c r="D7" s="33"/>
-      <c r="E7" s="22" t="s">
+      <c r="E7" s="30" t="s">
         <v>1355</v>
       </c>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+      <c r="J7" s="30"/>
+      <c r="K7" s="30"/>
+      <c r="L7" s="30"/>
     </row>
     <row r="8" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
@@ -21004,16 +21012,16 @@
       <c r="B8" s="33"/>
       <c r="C8" s="33"/>
       <c r="D8" s="33"/>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="30" t="s">
         <v>1356</v>
       </c>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="22"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="30"/>
     </row>
     <row r="9" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
@@ -21022,16 +21030,16 @@
       <c r="B9" s="33"/>
       <c r="C9" s="33"/>
       <c r="D9" s="33"/>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="30" t="s">
         <v>1357</v>
       </c>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="22"/>
-      <c r="L9" s="22"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30"/>
+      <c r="K9" s="30"/>
+      <c r="L9" s="30"/>
     </row>
     <row r="10" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
@@ -21040,16 +21048,16 @@
       <c r="B10" s="33"/>
       <c r="C10" s="33"/>
       <c r="D10" s="33"/>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="30" t="s">
         <v>1254</v>
       </c>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="22"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="12" spans="1:22" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
@@ -22210,6 +22218,12 @@
   </sheetData>
   <autoFilter ref="A12:V28" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
   <mergeCells count="14">
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:L4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E5:L5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:L6"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="E10:L10"/>
     <mergeCell ref="A7:D7"/>
@@ -22218,12 +22232,6 @@
     <mergeCell ref="E8:L8"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="E9:L9"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:L4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:L5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="E6:L6"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="U13:U28" xr:uid="{00000000-0002-0000-0700-000000000000}">
@@ -22278,16 +22286,16 @@
       <c r="B4" s="33"/>
       <c r="C4" s="33"/>
       <c r="D4" s="33"/>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="30" t="s">
         <v>1453</v>
       </c>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
     </row>
     <row r="5" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
@@ -22296,16 +22304,16 @@
       <c r="B5" s="33"/>
       <c r="C5" s="33"/>
       <c r="D5" s="33"/>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="30" t="s">
         <v>1454</v>
       </c>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="30"/>
+      <c r="L5" s="30"/>
     </row>
     <row r="6" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
@@ -22314,16 +22322,16 @@
       <c r="B6" s="33"/>
       <c r="C6" s="33"/>
       <c r="D6" s="33"/>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="30" t="s">
         <v>1455</v>
       </c>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="30"/>
+      <c r="K6" s="30"/>
+      <c r="L6" s="30"/>
     </row>
     <row r="7" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
@@ -22332,16 +22340,16 @@
       <c r="B7" s="33"/>
       <c r="C7" s="33"/>
       <c r="D7" s="33"/>
-      <c r="E7" s="22" t="s">
+      <c r="E7" s="30" t="s">
         <v>1456</v>
       </c>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+      <c r="J7" s="30"/>
+      <c r="K7" s="30"/>
+      <c r="L7" s="30"/>
     </row>
     <row r="8" spans="1:22" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
@@ -22350,16 +22358,16 @@
       <c r="B8" s="33"/>
       <c r="C8" s="33"/>
       <c r="D8" s="33"/>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="30" t="s">
         <v>1457</v>
       </c>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="22"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="30"/>
     </row>
     <row r="9" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
@@ -22368,16 +22376,16 @@
       <c r="B9" s="33"/>
       <c r="C9" s="33"/>
       <c r="D9" s="33"/>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="30" t="s">
         <v>1458</v>
       </c>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="22"/>
-      <c r="L9" s="22"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30"/>
+      <c r="K9" s="30"/>
+      <c r="L9" s="30"/>
     </row>
     <row r="10" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
@@ -22386,16 +22394,16 @@
       <c r="B10" s="33"/>
       <c r="C10" s="33"/>
       <c r="D10" s="33"/>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="30" t="s">
         <v>1254</v>
       </c>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="22"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="12" spans="1:22" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
@@ -23556,6 +23564,12 @@
   </sheetData>
   <autoFilter ref="A12:V28" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
   <mergeCells count="14">
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:L4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E5:L5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:L6"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="E10:L10"/>
     <mergeCell ref="A7:D7"/>
@@ -23564,12 +23578,6 @@
     <mergeCell ref="E8:L8"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="E9:L9"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:L4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:L5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="E6:L6"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="U13:U28" xr:uid="{00000000-0002-0000-0800-000000000000}">

</xml_diff>